<commit_message>
should have 80% to PIH
</commit_message>
<xml_diff>
--- a/data/surveillance_costing.xlsx
+++ b/data/surveillance_costing.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/briday/Desktop/study_stats/D2P_project/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AEBE1F90-18A4-834C-A989-0D959ADDF5EB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{951CE3B7-C460-EC47-B563-ED253C57557E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="24340" windowHeight="12740" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="24340" windowHeight="12740" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="README" sheetId="1" r:id="rId1"/>
@@ -147,9 +147,6 @@
     <t>Poisons information specialist</t>
   </si>
   <si>
-    <t>Pesticide is ~15% of PIH call volume (1,158 of ~7,700 clinician-initiated calls).</t>
-  </si>
-  <si>
     <t>DoH pharmacy OSD 2024; PIH 2023 report</t>
   </si>
   <si>
@@ -337,6 +334,9 @@
   </si>
   <si>
     <t xml:space="preserve">increases number of SMSs to be sent out when increase in coordination. </t>
+  </si>
+  <si>
+    <t>Pesticide is ~80% of PIH call volume (1,158 of ~7,700 clinician-initiated calls).</t>
   </si>
 </sst>
 </file>
@@ -800,16 +800,16 @@
         <v>16</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>80</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>82</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>83</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>21</v>
@@ -823,7 +823,7 @@
         <v>23</v>
       </c>
       <c r="B2" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="C2">
         <v>1013</v>
@@ -835,10 +835,10 @@
         <v>0.84</v>
       </c>
       <c r="F2" t="s">
+        <v>84</v>
+      </c>
+      <c r="G2" t="s">
         <v>85</v>
-      </c>
-      <c r="G2" t="s">
-        <v>86</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.2">
@@ -846,7 +846,7 @@
         <v>33</v>
       </c>
       <c r="B3" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="C3">
         <v>17000</v>
@@ -858,18 +858,18 @@
         <v>15.04</v>
       </c>
       <c r="F3" t="s">
+        <v>87</v>
+      </c>
+      <c r="G3" t="s">
         <v>88</v>
-      </c>
-      <c r="G3" t="s">
-        <v>89</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B4" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="C4">
         <v>10626</v>
@@ -881,10 +881,10 @@
         <v>100</v>
       </c>
       <c r="F4" t="s">
+        <v>90</v>
+      </c>
+      <c r="G4" t="s">
         <v>91</v>
-      </c>
-      <c r="G4" t="s">
-        <v>92</v>
       </c>
     </row>
   </sheetData>
@@ -948,10 +948,10 @@
         <v>624000</v>
       </c>
       <c r="F2" t="s">
+        <v>98</v>
+      </c>
+      <c r="G2" t="s">
         <v>35</v>
-      </c>
-      <c r="G2" t="s">
-        <v>36</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.2">
@@ -980,10 +980,10 @@
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
+        <v>40</v>
+      </c>
+      <c r="B4" t="s">
         <v>41</v>
-      </c>
-      <c r="B4" t="s">
-        <v>42</v>
       </c>
       <c r="C4" s="2">
         <v>750000</v>
@@ -996,10 +996,10 @@
         <v>75000</v>
       </c>
       <c r="F4" t="s">
+        <v>42</v>
+      </c>
+      <c r="G4" t="s">
         <v>43</v>
-      </c>
-      <c r="G4" t="s">
-        <v>44</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.2">
@@ -1007,7 +1007,7 @@
         <v>33</v>
       </c>
       <c r="B5" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C5" s="2">
         <v>1300000</v>
@@ -1020,18 +1020,18 @@
         <v>65000</v>
       </c>
       <c r="F5" t="s">
+        <v>37</v>
+      </c>
+      <c r="G5" t="s">
         <v>38</v>
-      </c>
-      <c r="G5" t="s">
-        <v>39</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B6" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C6" s="2">
         <v>850000</v>
@@ -1044,10 +1044,10 @@
         <v>42500</v>
       </c>
       <c r="F6" t="s">
+        <v>45</v>
+      </c>
+      <c r="G6" t="s">
         <v>46</v>
-      </c>
-      <c r="G6" t="s">
-        <v>47</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.2">
@@ -1131,13 +1131,13 @@
         <v>16</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" s="3" t="s">
         <v>49</v>
-      </c>
-      <c r="D1" s="3" t="s">
-        <v>50</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>20</v>
@@ -1149,7 +1149,7 @@
         <v>22</v>
       </c>
       <c r="H1" s="7" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.2">
@@ -1157,7 +1157,7 @@
         <v>23</v>
       </c>
       <c r="B2" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C2" s="2">
         <v>180000</v>
@@ -1170,10 +1170,10 @@
         <v>180000</v>
       </c>
       <c r="F2" t="s">
+        <v>51</v>
+      </c>
+      <c r="G2" t="s">
         <v>52</v>
-      </c>
-      <c r="G2" t="s">
-        <v>53</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.2">
@@ -1181,7 +1181,7 @@
         <v>23</v>
       </c>
       <c r="B3" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C3" s="2">
         <v>0.15</v>
@@ -1195,13 +1195,13 @@
         <v>3000</v>
       </c>
       <c r="F3" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="G3" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="H3" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.2">
@@ -1209,7 +1209,7 @@
         <v>23</v>
       </c>
       <c r="B4" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C4" s="2">
         <v>18000</v>
@@ -1222,10 +1222,10 @@
         <v>18000</v>
       </c>
       <c r="F4" t="s">
+        <v>56</v>
+      </c>
+      <c r="G4" t="s">
         <v>57</v>
-      </c>
-      <c r="G4" t="s">
-        <v>58</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.2">
@@ -1233,7 +1233,7 @@
         <v>33</v>
       </c>
       <c r="B5" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="C5" s="2">
         <v>120000</v>
@@ -1246,10 +1246,10 @@
         <v>120000</v>
       </c>
       <c r="F5" t="s">
+        <v>59</v>
+      </c>
+      <c r="G5" t="s">
         <v>60</v>
-      </c>
-      <c r="G5" t="s">
-        <v>61</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.2">
@@ -1257,7 +1257,7 @@
         <v>33</v>
       </c>
       <c r="B6" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C6" s="2">
         <v>85000</v>
@@ -1270,10 +1270,10 @@
         <v>72250</v>
       </c>
       <c r="F6" t="s">
+        <v>62</v>
+      </c>
+      <c r="G6" t="s">
         <v>63</v>
-      </c>
-      <c r="G6" t="s">
-        <v>64</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.2">
@@ -1281,7 +1281,7 @@
         <v>33</v>
       </c>
       <c r="B7" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="C7" s="2">
         <v>42000</v>
@@ -1294,18 +1294,18 @@
         <v>42000</v>
       </c>
       <c r="F7" t="s">
+        <v>65</v>
+      </c>
+      <c r="G7" t="s">
         <v>66</v>
-      </c>
-      <c r="G7" t="s">
-        <v>67</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B8" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C8" s="2">
         <v>90.22</v>
@@ -1318,18 +1318,18 @@
         <v>958677.72</v>
       </c>
       <c r="F8" t="s">
+        <v>68</v>
+      </c>
+      <c r="G8" t="s">
         <v>69</v>
-      </c>
-      <c r="G8" t="s">
-        <v>70</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B9" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C9" s="2">
         <v>180000</v>
@@ -1342,18 +1342,18 @@
         <v>180000</v>
       </c>
       <c r="F9" t="s">
+        <v>71</v>
+      </c>
+      <c r="G9" t="s">
         <v>72</v>
-      </c>
-      <c r="G9" t="s">
-        <v>73</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B10" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="C10" s="2">
         <v>25</v>
@@ -1366,18 +1366,18 @@
         <v>265650</v>
       </c>
       <c r="F10" t="s">
+        <v>74</v>
+      </c>
+      <c r="G10" t="s">
         <v>75</v>
-      </c>
-      <c r="G10" t="s">
-        <v>76</v>
       </c>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B11" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C11" s="2">
         <v>240000</v>
@@ -1390,10 +1390,10 @@
         <v>240000</v>
       </c>
       <c r="F11" t="s">
+        <v>77</v>
+      </c>
+      <c r="G11" t="s">
         <v>78</v>
-      </c>
-      <c r="G11" t="s">
-        <v>79</v>
       </c>
     </row>
   </sheetData>
@@ -1409,7 +1409,7 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B1" s="6">
         <f>SUM(personnel!E2:E8)</f>
@@ -1418,7 +1418,7 @@
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="B2" s="6">
         <f>SUM(system!E2:E11)</f>
@@ -1427,7 +1427,7 @@
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="B3" s="6">
         <f xml:space="preserve"> SUM(B1:B2)</f>

</xml_diff>